<commit_message>
Update Cash_flows_statement '24-'14 cleaned.xlsx
</commit_message>
<xml_diff>
--- a/Edgar_Tools/Cash_flows_statement '24-'14 cleaned.xlsx
+++ b/Edgar_Tools/Cash_flows_statement '24-'14 cleaned.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vermouth/Documents/GitHub/Data-Analysis-Projects/Edgar_Tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDD1D617-192B-D046-90E0-7C39A54AFEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{030CD60F-4B37-8242-9103-2AA6326339F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{9C34E956-EC8A-894F-96DF-C3655B97DAEA}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{9C34E956-EC8A-894F-96DF-C3655B97DAEA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="cleaned" sheetId="2" r:id="rId2"/>
+    <sheet name="copy from Py" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="704" uniqueCount="368">
   <si>
     <t>label</t>
   </si>
@@ -201,13 +202,952 @@
   </si>
   <si>
     <t>PaymentsForStrategicInvestments</t>
+  </si>
+  <si>
+    <t>Operating activities:</t>
+  </si>
+  <si>
+    <t>Net Income</t>
+  </si>
+  <si>
+    <t>Adjustments to reconcile net income to cash generated by operating activities:</t>
+  </si>
+  <si>
+    <t>Depreciation and amortization</t>
+  </si>
+  <si>
+    <t>Share-based compensation expense</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Changes in operating assets and liabilities:</t>
+  </si>
+  <si>
+    <t>Accounts receivable, net</t>
+  </si>
+  <si>
+    <t>Vendor non-trade receivables</t>
+  </si>
+  <si>
+    <t>Other current and non-current assets</t>
+  </si>
+  <si>
+    <t>Accounts payable</t>
+  </si>
+  <si>
+    <t>Other current and non-current liabilities</t>
+  </si>
+  <si>
+    <t>Net Cash from Operating Activities</t>
+  </si>
+  <si>
+    <t>Investing activities:</t>
+  </si>
+  <si>
+    <t>Purchases of marketable securities</t>
+  </si>
+  <si>
+    <t>Proceeds from Maturities, Prepayments and Calls of Securities</t>
+  </si>
+  <si>
+    <t>Proceeds from Sale of Debt Securities,</t>
+  </si>
+  <si>
+    <t>Payments for Property, Plant and Equipment</t>
+  </si>
+  <si>
+    <t>Net Cash from Investing Activities</t>
+  </si>
+  <si>
+    <t>Financing activities:</t>
+  </si>
+  <si>
+    <t>Tax Withholding for Share-Based Compensation</t>
+  </si>
+  <si>
+    <t>Payments of Dividends</t>
+  </si>
+  <si>
+    <t>Repurchases of common stock</t>
+  </si>
+  <si>
+    <t>Proceeds from Issuance of Long-Term Debt</t>
+  </si>
+  <si>
+    <t>Repayments of term debt</t>
+  </si>
+  <si>
+    <t>Proceeds from (Repayments of) Commercial Paper</t>
+  </si>
+  <si>
+    <t>Net Cash from Financing Activities</t>
+  </si>
+  <si>
+    <t>Net Change in Cash</t>
+  </si>
+  <si>
+    <t>Supplemental cash flow disclosure:</t>
+  </si>
+  <si>
+    <t>Income Tax Expense</t>
+  </si>
+  <si>
+    <t>Sep 25, 2021</t>
+  </si>
+  <si>
+    <t>Sep 26, 2020</t>
+  </si>
+  <si>
+    <t>Sep 28, 2019</t>
+  </si>
+  <si>
+    <t>Cash, cash equivalents and restricted cash, ending balances</t>
+  </si>
+  <si>
+    <t>$94,680</t>
+  </si>
+  <si>
+    <t>$57,411</t>
+  </si>
+  <si>
+    <t>$55,256</t>
+  </si>
+  <si>
+    <t>$11,284</t>
+  </si>
+  <si>
+    <t>$11,056</t>
+  </si>
+  <si>
+    <t>$12,547</t>
+  </si>
+  <si>
+    <t>$7,906</t>
+  </si>
+  <si>
+    <t>$6,829</t>
+  </si>
+  <si>
+    <t>$6,068</t>
+  </si>
+  <si>
+    <t>Deferred income tax benefit</t>
+  </si>
+  <si>
+    <t>$6,917</t>
+  </si>
+  <si>
+    <t>$245</t>
+  </si>
+  <si>
+    <t>$1,553</t>
+  </si>
+  <si>
+    <t>$2,931</t>
+  </si>
+  <si>
+    <t>$873</t>
+  </si>
+  <si>
+    <t>$12,326</t>
+  </si>
+  <si>
+    <t>Deferred revenue</t>
+  </si>
+  <si>
+    <t>$1,676</t>
+  </si>
+  <si>
+    <t>$2,081</t>
+  </si>
+  <si>
+    <t>$5,799</t>
+  </si>
+  <si>
+    <t>$8,916</t>
+  </si>
+  <si>
+    <t>$104,038</t>
+  </si>
+  <si>
+    <t>$80,674</t>
+  </si>
+  <si>
+    <t>$69,391</t>
+  </si>
+  <si>
+    <t>$59,023</t>
+  </si>
+  <si>
+    <t>$69,918</t>
+  </si>
+  <si>
+    <t>$40,102</t>
+  </si>
+  <si>
+    <t>$47,460</t>
+  </si>
+  <si>
+    <t>$50,473</t>
+  </si>
+  <si>
+    <t>$56,988</t>
+  </si>
+  <si>
+    <t>Payments to Acquire Businesses</t>
+  </si>
+  <si>
+    <t>Purchases of non-marketable securities</t>
+  </si>
+  <si>
+    <t>Proceeds from Sale and Maturity of Other Investments</t>
+  </si>
+  <si>
+    <t>$387</t>
+  </si>
+  <si>
+    <t>$92</t>
+  </si>
+  <si>
+    <t>$1,634</t>
+  </si>
+  <si>
+    <t>$45,896</t>
+  </si>
+  <si>
+    <t>Proceeds from Issuance of Common Stock</t>
+  </si>
+  <si>
+    <t>$1,105</t>
+  </si>
+  <si>
+    <t>$880</t>
+  </si>
+  <si>
+    <t>$781</t>
+  </si>
+  <si>
+    <t>$20,393</t>
+  </si>
+  <si>
+    <t>$16,091</t>
+  </si>
+  <si>
+    <t>$6,963</t>
+  </si>
+  <si>
+    <t>$1,022</t>
+  </si>
+  <si>
+    <t>$24,311</t>
+  </si>
+  <si>
+    <t>$25,385</t>
+  </si>
+  <si>
+    <t>$9,501</t>
+  </si>
+  <si>
+    <t>$15,263</t>
+  </si>
+  <si>
+    <t>Cash paid for interest</t>
+  </si>
+  <si>
+    <t>Sep 29, 2018</t>
+  </si>
+  <si>
+    <t>Sep 30, 2017</t>
+  </si>
+  <si>
+    <t>Sep 24, 2016</t>
+  </si>
+  <si>
+    <t>Cash and Cash Equivalents</t>
+  </si>
+  <si>
+    <t>$59,531</t>
+  </si>
+  <si>
+    <t>$48,351</t>
+  </si>
+  <si>
+    <t>$45,687</t>
+  </si>
+  <si>
+    <t>$10,903</t>
+  </si>
+  <si>
+    <t>$10,157</t>
+  </si>
+  <si>
+    <t>$10,505</t>
+  </si>
+  <si>
+    <t>$5,340</t>
+  </si>
+  <si>
+    <t>$4,840</t>
+  </si>
+  <si>
+    <t>$4,210</t>
+  </si>
+  <si>
+    <t>Deferred income tax expense/(benefit)</t>
+  </si>
+  <si>
+    <t>$5,966</t>
+  </si>
+  <si>
+    <t>$4,938</t>
+  </si>
+  <si>
+    <t>$486</t>
+  </si>
+  <si>
+    <t>$527</t>
+  </si>
+  <si>
+    <t>$828</t>
+  </si>
+  <si>
+    <t>$217</t>
+  </si>
+  <si>
+    <t>$1,055</t>
+  </si>
+  <si>
+    <t>$9,175</t>
+  </si>
+  <si>
+    <t>$8,966</t>
+  </si>
+  <si>
+    <t>$2,117</t>
+  </si>
+  <si>
+    <t>$38,490</t>
+  </si>
+  <si>
+    <t>$1,125</t>
+  </si>
+  <si>
+    <t>$77,434</t>
+  </si>
+  <si>
+    <t>$64,225</t>
+  </si>
+  <si>
+    <t>$66,231</t>
+  </si>
+  <si>
+    <t>$55,881</t>
+  </si>
+  <si>
+    <t>$31,775</t>
+  </si>
+  <si>
+    <t>$21,258</t>
+  </si>
+  <si>
+    <t>Proceeds from sales of marketable securities</t>
+  </si>
+  <si>
+    <t>$47,838</t>
+  </si>
+  <si>
+    <t>$94,564</t>
+  </si>
+  <si>
+    <t>$90,536</t>
+  </si>
+  <si>
+    <t>$353</t>
+  </si>
+  <si>
+    <t>$126</t>
+  </si>
+  <si>
+    <t>$16,066</t>
+  </si>
+  <si>
+    <t>$669</t>
+  </si>
+  <si>
+    <t>$555</t>
+  </si>
+  <si>
+    <t>$495</t>
+  </si>
+  <si>
+    <t>$6,969</t>
+  </si>
+  <si>
+    <t>$28,662</t>
+  </si>
+  <si>
+    <t>$24,954</t>
+  </si>
+  <si>
+    <t>$3,852</t>
+  </si>
+  <si>
+    <t>$5,624</t>
+  </si>
+  <si>
+    <t>$10,417</t>
+  </si>
+  <si>
+    <t>$11,591</t>
+  </si>
+  <si>
+    <t>$10,444</t>
+  </si>
+  <si>
+    <t>$3,022</t>
+  </si>
+  <si>
+    <t>$2,092</t>
+  </si>
+  <si>
+    <t>$1,316</t>
+  </si>
+  <si>
+    <t>Sep 26, 2015</t>
+  </si>
+  <si>
+    <t>Sep 27, 2014</t>
+  </si>
+  <si>
+    <t>$53,394</t>
+  </si>
+  <si>
+    <t>$39,510</t>
+  </si>
+  <si>
+    <t>$11,257</t>
+  </si>
+  <si>
+    <t>$7,946</t>
+  </si>
+  <si>
+    <t>$3,586</t>
+  </si>
+  <si>
+    <t>$2,863</t>
+  </si>
+  <si>
+    <t>Deferred income tax expense</t>
+  </si>
+  <si>
+    <t>$1,382</t>
+  </si>
+  <si>
+    <t>$2,347</t>
+  </si>
+  <si>
+    <t>$611</t>
+  </si>
+  <si>
+    <t>$167</t>
+  </si>
+  <si>
+    <t>$5,400</t>
+  </si>
+  <si>
+    <t>$5,938</t>
+  </si>
+  <si>
+    <t>$1,042</t>
+  </si>
+  <si>
+    <t>$1,460</t>
+  </si>
+  <si>
+    <t>$8,746</t>
+  </si>
+  <si>
+    <t>$6,010</t>
+  </si>
+  <si>
+    <t>$81,266</t>
+  </si>
+  <si>
+    <t>$59,713</t>
+  </si>
+  <si>
+    <t>$14,538</t>
+  </si>
+  <si>
+    <t>$18,810</t>
+  </si>
+  <si>
+    <t>$107,447</t>
+  </si>
+  <si>
+    <t>$189,301</t>
+  </si>
+  <si>
+    <t>Payments for acquisition of intangible assets</t>
+  </si>
+  <si>
+    <t>$16</t>
+  </si>
+  <si>
+    <t>$543</t>
+  </si>
+  <si>
+    <t>$730</t>
+  </si>
+  <si>
+    <t>Excess tax benefits from equity awards</t>
+  </si>
+  <si>
+    <t>$749</t>
+  </si>
+  <si>
+    <t>$739</t>
+  </si>
+  <si>
+    <t>Dividends and dividend equivalents paid</t>
+  </si>
+  <si>
+    <t>Repurchase of common stock</t>
+  </si>
+  <si>
+    <t>$27,114</t>
+  </si>
+  <si>
+    <t>$11,960</t>
+  </si>
+  <si>
+    <t>$2,191</t>
+  </si>
+  <si>
+    <t>$6,306</t>
+  </si>
+  <si>
+    <t>$7,276</t>
+  </si>
+  <si>
+    <t>$13,252</t>
+  </si>
+  <si>
+    <t>$10,026</t>
+  </si>
+  <si>
+    <t>$514</t>
+  </si>
+  <si>
+    <t>$339</t>
+  </si>
+  <si>
+    <t>-$4,774</t>
+  </si>
+  <si>
+    <t>-$215</t>
+  </si>
+  <si>
+    <t>-$340</t>
+  </si>
+  <si>
+    <t>-$32,590</t>
+  </si>
+  <si>
+    <t>-$147</t>
+  </si>
+  <si>
+    <t>-$97</t>
+  </si>
+  <si>
+    <t>-$652</t>
+  </si>
+  <si>
+    <t>-$444</t>
+  </si>
+  <si>
+    <t>-$166</t>
+  </si>
+  <si>
+    <t>-$4,232</t>
+  </si>
+  <si>
+    <t>-$10,125</t>
+  </si>
+  <si>
+    <t>-$5,322</t>
+  </si>
+  <si>
+    <t>-$2,093</t>
+  </si>
+  <si>
+    <t>-$238</t>
+  </si>
+  <si>
+    <t>-$76</t>
+  </si>
+  <si>
+    <t>-$2,642</t>
+  </si>
+  <si>
+    <t>-$127</t>
+  </si>
+  <si>
+    <t>-$289</t>
+  </si>
+  <si>
+    <t>-$2,723</t>
+  </si>
+  <si>
+    <t>-$3,735</t>
+  </si>
+  <si>
+    <t>-$2,220</t>
+  </si>
+  <si>
+    <t>-$3,903</t>
+  </si>
+  <si>
+    <t>-$8,010</t>
+  </si>
+  <si>
+    <t>-$4,254</t>
+  </si>
+  <si>
+    <t>-$51</t>
+  </si>
+  <si>
+    <t>-$179</t>
+  </si>
+  <si>
+    <t>-$8,042</t>
+  </si>
+  <si>
+    <t>-$9,588</t>
+  </si>
+  <si>
+    <t>-$423</t>
+  </si>
+  <si>
+    <t>-$5,318</t>
+  </si>
+  <si>
+    <t>-$4,062</t>
+  </si>
+  <si>
+    <t>-$1,923</t>
+  </si>
+  <si>
+    <t>-$625</t>
+  </si>
+  <si>
+    <t>-$44</t>
+  </si>
+  <si>
+    <t>-$626</t>
+  </si>
+  <si>
+    <t>-$1,554</t>
+  </si>
+  <si>
+    <t>-$4,700</t>
+  </si>
+  <si>
+    <t>-$1,906</t>
+  </si>
+  <si>
+    <t>-$166,402</t>
+  </si>
+  <si>
+    <t>-$217,128</t>
+  </si>
+  <si>
+    <t>-$109,558</t>
+  </si>
+  <si>
+    <t>-$114,938</t>
+  </si>
+  <si>
+    <t>-$39,630</t>
+  </si>
+  <si>
+    <t>-$71,356</t>
+  </si>
+  <si>
+    <t>-$159,486</t>
+  </si>
+  <si>
+    <t>-$142,428</t>
+  </si>
+  <si>
+    <t>-$343</t>
+  </si>
+  <si>
+    <t>-$3,765</t>
+  </si>
+  <si>
+    <t>-$11,085</t>
+  </si>
+  <si>
+    <t>-$7,309</t>
+  </si>
+  <si>
+    <t>-$10,495</t>
+  </si>
+  <si>
+    <t>-$13,313</t>
+  </si>
+  <si>
+    <t>-$12,451</t>
+  </si>
+  <si>
+    <t>-$12,734</t>
+  </si>
+  <si>
+    <t>-$11,247</t>
+  </si>
+  <si>
+    <t>-$9,571</t>
+  </si>
+  <si>
+    <t>-$33</t>
+  </si>
+  <si>
+    <t>-$1,524</t>
+  </si>
+  <si>
+    <t>-$624</t>
+  </si>
+  <si>
+    <t>-$721</t>
+  </si>
+  <si>
+    <t>-$329</t>
+  </si>
+  <si>
+    <t>-$297</t>
+  </si>
+  <si>
+    <t>-$241</t>
+  </si>
+  <si>
+    <t>-$242</t>
+  </si>
+  <si>
+    <t>-$131</t>
+  </si>
+  <si>
+    <t>-$210</t>
+  </si>
+  <si>
+    <t>-$1,001</t>
+  </si>
+  <si>
+    <t>-$1,871</t>
+  </si>
+  <si>
+    <t>-$521</t>
+  </si>
+  <si>
+    <t>-$1,388</t>
+  </si>
+  <si>
+    <t>-$26</t>
+  </si>
+  <si>
+    <t>-$56,274</t>
+  </si>
+  <si>
+    <t>-$22,579</t>
+  </si>
+  <si>
+    <t>-$608</t>
+  </si>
+  <si>
+    <t>-$791</t>
+  </si>
+  <si>
+    <t>-$1,078</t>
+  </si>
+  <si>
+    <t>-$745</t>
+  </si>
+  <si>
+    <t>-$124</t>
+  </si>
+  <si>
+    <t>-$924</t>
+  </si>
+  <si>
+    <t>-$14,545</t>
+  </si>
+  <si>
+    <t>-$4,289</t>
+  </si>
+  <si>
+    <t>-$46,446</t>
+  </si>
+  <si>
+    <t>-$45,977</t>
+  </si>
+  <si>
+    <t>-$1,499</t>
+  </si>
+  <si>
+    <t>-$1,158</t>
+  </si>
+  <si>
+    <t>-$6,556</t>
+  </si>
+  <si>
+    <t>-$3,634</t>
+  </si>
+  <si>
+    <t>-$2,817</t>
+  </si>
+  <si>
+    <t>-$2,527</t>
+  </si>
+  <si>
+    <t>-$1,874</t>
+  </si>
+  <si>
+    <t>-$1,570</t>
+  </si>
+  <si>
+    <t>-$11,561</t>
+  </si>
+  <si>
+    <t>-$11,126</t>
+  </si>
+  <si>
+    <t>-$14,467</t>
+  </si>
+  <si>
+    <t>-$14,081</t>
+  </si>
+  <si>
+    <t>-$14,119</t>
+  </si>
+  <si>
+    <t>-$13,712</t>
+  </si>
+  <si>
+    <t>-$12,769</t>
+  </si>
+  <si>
+    <t>-$12,150</t>
+  </si>
+  <si>
+    <t>-$35,253</t>
+  </si>
+  <si>
+    <t>-$45,000</t>
+  </si>
+  <si>
+    <t>-$85,971</t>
+  </si>
+  <si>
+    <t>-$72,358</t>
+  </si>
+  <si>
+    <t>-$66,897</t>
+  </si>
+  <si>
+    <t>-$72,738</t>
+  </si>
+  <si>
+    <t>-$32,900</t>
+  </si>
+  <si>
+    <t>-$29,722</t>
+  </si>
+  <si>
+    <t>-$8,750</t>
+  </si>
+  <si>
+    <t>-$12,629</t>
+  </si>
+  <si>
+    <t>-$8,805</t>
+  </si>
+  <si>
+    <t>-$6,500</t>
+  </si>
+  <si>
+    <t>-$3,500</t>
+  </si>
+  <si>
+    <t>-$2,500</t>
+  </si>
+  <si>
+    <t>-$17,716</t>
+  </si>
+  <si>
+    <t>-$37,549</t>
+  </si>
+  <si>
+    <t>-$963</t>
+  </si>
+  <si>
+    <t>-$5,977</t>
+  </si>
+  <si>
+    <t>-$37</t>
+  </si>
+  <si>
+    <t>-$397</t>
+  </si>
+  <si>
+    <t>-$415</t>
+  </si>
+  <si>
+    <t>-$129</t>
+  </si>
+  <si>
+    <t>-$126</t>
+  </si>
+  <si>
+    <t>-$105</t>
+  </si>
+  <si>
+    <t>-$87,876</t>
+  </si>
+  <si>
+    <t>-$17,974</t>
+  </si>
+  <si>
+    <t>-$20,890</t>
+  </si>
+  <si>
+    <t>-$93,353</t>
+  </si>
+  <si>
+    <t>-$86,820</t>
+  </si>
+  <si>
+    <t>-$90,976</t>
+  </si>
+  <si>
+    <t>-$195</t>
+  </si>
+  <si>
+    <t>-$636</t>
+  </si>
+  <si>
+    <t>-$3,860</t>
+  </si>
+  <si>
+    <t>-$10,435</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -238,6 +1178,18 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -295,7 +1247,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -308,6 +1260,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4495,4 +5449,1424 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4138336-DEE9-674B-91C0-778671718B39}">
+  <dimension ref="A1:M42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="69.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="10"/>
+      <c r="B1" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" s="10"/>
+      <c r="M3" s="10"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" s="10"/>
+      <c r="F4" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="J4" s="10"/>
+      <c r="K4" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="J6" s="10"/>
+      <c r="K6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="M6" s="11" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" s="10"/>
+      <c r="F7" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="J7" s="10"/>
+      <c r="K7" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="L7" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="M7" s="11" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="E8" s="10"/>
+      <c r="F8" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="J8" s="10"/>
+      <c r="K8" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="L8" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="E9" s="10"/>
+      <c r="F9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="J9" s="10"/>
+      <c r="K9" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="L10" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="M10" s="11" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="J11" s="10"/>
+      <c r="K11" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="L11" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="M11" s="11" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="E12" s="10"/>
+      <c r="F12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="J12" s="10"/>
+      <c r="K12" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="L12" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A13" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="J13" s="10"/>
+      <c r="K13" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A14" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="E14" s="10"/>
+      <c r="F14" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="J14" s="10"/>
+      <c r="K14" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="L14" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A15" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="J15" s="10"/>
+      <c r="K15" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="L15" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="M15" s="11" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="E16" s="10"/>
+      <c r="F16" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>268</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>270</v>
+      </c>
+      <c r="J16" s="10"/>
+      <c r="K16" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="J17" s="10"/>
+      <c r="K17" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="E18" s="10"/>
+      <c r="F18" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="J18" s="10"/>
+      <c r="K18" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>277</v>
+      </c>
+      <c r="E20" s="10"/>
+      <c r="F20" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>280</v>
+      </c>
+      <c r="J20" s="10"/>
+      <c r="K20" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="L20" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="E21" s="10"/>
+      <c r="F21" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="J21" s="10"/>
+      <c r="K21" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="L21" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="M21" s="11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="10"/>
+      <c r="F22" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="J22" s="10"/>
+      <c r="K22" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="L22" s="11" t="s">
+        <v>281</v>
+      </c>
+      <c r="M22" s="11" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>283</v>
+      </c>
+      <c r="C23" s="11" t="s">
+        <v>284</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>285</v>
+      </c>
+      <c r="E23" s="10"/>
+      <c r="F23" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>287</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="J23" s="10"/>
+      <c r="K23" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="L23" s="11" t="s">
+        <v>289</v>
+      </c>
+      <c r="M23" s="11" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>292</v>
+      </c>
+      <c r="D24" s="11" t="s">
+        <v>293</v>
+      </c>
+      <c r="E24" s="10"/>
+      <c r="F24" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>296</v>
+      </c>
+      <c r="J24" s="10"/>
+      <c r="K24" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="L24" s="11" t="s">
+        <v>297</v>
+      </c>
+      <c r="M24" s="11" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="E25" s="10"/>
+      <c r="F25" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>304</v>
+      </c>
+      <c r="J25" s="10"/>
+      <c r="K25" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="L25" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="M25" s="11" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E26" s="10"/>
+      <c r="F26" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="L26" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="M26" s="11" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="E27" s="10"/>
+      <c r="F27" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="J27" s="10"/>
+      <c r="K27" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="L27" s="10"/>
+      <c r="M27" s="10"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A28" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="C28" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="E28" s="10"/>
+      <c r="F28" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="J28" s="10"/>
+      <c r="K28" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="L28" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="M28" s="11" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A29" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" s="10"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="L29" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="M29" s="11" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A30" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="E30" s="10"/>
+      <c r="F30" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="J30" s="10"/>
+      <c r="K30" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="L30" s="11" t="s">
+        <v>318</v>
+      </c>
+      <c r="M30" s="11" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A31" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>321</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>322</v>
+      </c>
+      <c r="E31" s="10"/>
+      <c r="F31" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>324</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>325</v>
+      </c>
+      <c r="J31" s="10"/>
+      <c r="K31" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="L31" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="M31" s="11" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A32" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>330</v>
+      </c>
+      <c r="E32" s="10"/>
+      <c r="F32" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>333</v>
+      </c>
+      <c r="J32" s="10"/>
+      <c r="K32" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="L32" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="M32" s="11" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A33" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>338</v>
+      </c>
+      <c r="E33" s="10"/>
+      <c r="F33" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>339</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>341</v>
+      </c>
+      <c r="J33" s="10"/>
+      <c r="K33" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="L33" s="11" t="s">
+        <v>226</v>
+      </c>
+      <c r="M33" s="11" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A34" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E34" s="10"/>
+      <c r="F34" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G34" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="J34" s="10"/>
+      <c r="K34" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L34" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="M34" s="11" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A35" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>342</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>343</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>344</v>
+      </c>
+      <c r="E35" s="10"/>
+      <c r="F35" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>345</v>
+      </c>
+      <c r="H35" s="11" t="s">
+        <v>346</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="J35" s="10"/>
+      <c r="K35" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="L35" s="11" t="s">
+        <v>348</v>
+      </c>
+      <c r="M35" s="11" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>350</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>351</v>
+      </c>
+      <c r="E36" s="10"/>
+      <c r="F36" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="G36" s="11" t="s">
+        <v>352</v>
+      </c>
+      <c r="H36" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="I36" s="11" t="s">
+        <v>353</v>
+      </c>
+      <c r="J36" s="10"/>
+      <c r="K36" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="L36" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="M36" s="11" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>355</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>356</v>
+      </c>
+      <c r="D37" s="11" t="s">
+        <v>357</v>
+      </c>
+      <c r="E37" s="10"/>
+      <c r="F37" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="I37" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="J37" s="10"/>
+      <c r="K37" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A38" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>362</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="E38" s="10"/>
+      <c r="F38" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="H38" s="11" t="s">
+        <v>364</v>
+      </c>
+      <c r="I38" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="J38" s="10"/>
+      <c r="K38" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="L38" s="10"/>
+      <c r="M38" s="10"/>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A39" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>367</v>
+      </c>
+      <c r="D39" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E39" s="10"/>
+      <c r="F39" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="L39" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="M39" s="11" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A40" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B40" s="10"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="L40" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="M40" s="11" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" s="10"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="G41" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="H41" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="I41" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+      <c r="M41" s="10"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="D42" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="E42" s="10"/>
+      <c r="F42" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="G42" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="H42" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="I42" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>